<commit_message>
make settings page functional
</commit_message>
<xml_diff>
--- a/examples/factura.xlsx
+++ b/examples/factura.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1901994F-E080-4BFD-86A6-3AD69EA3616A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6DA7E66-D9CE-43F8-8D87-227DACDEFB72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14775" yWindow="855" windowWidth="18900" windowHeight="19335" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Calle Principal, 123</t>
   </si>
@@ -44,9 +44,6 @@
     <t>Ocean View, MO 12345</t>
   </si>
   <si>
-    <t>FACTURAR A:</t>
-  </si>
-  <si>
     <t>CANT.</t>
   </si>
   <si>
@@ -56,26 +53,12 @@
     <t>interestingsite.com</t>
   </si>
   <si>
-    <t>Pedro Armijo</t>
-  </si>
-  <si>
-    <t>Fourth Coffee
-Calle Principal, 123
-Seattle, WA 12345</t>
-  </si>
-  <si>
-    <t>123-456-0134</t>
-  </si>
-  <si>
     <t>DESCRIPCIÓN</t>
   </si>
   <si>
     <t>N.º de factura:</t>
   </si>
   <si>
-    <t>ENVIAR A:</t>
-  </si>
-  <si>
     <t>PRECIO POR UNIDAD</t>
   </si>
   <si>
@@ -94,22 +77,28 @@
     <t>IVA</t>
   </si>
   <si>
-    <t xml:space="preserve">Juguetos </t>
-  </si>
-  <si>
-    <t>Lego Ducati Panigale V4 S 42202</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coches HotWheels </t>
-  </si>
-  <si>
-    <t>Puzzle Zoo 1000 Pcs.</t>
-  </si>
-  <si>
     <t>juguetos@info.es</t>
   </si>
   <si>
-    <t xml:space="preserve">CIF: </t>
+    <t>Eroski</t>
+  </si>
+  <si>
+    <t>Docena Huevos camperos</t>
+  </si>
+  <si>
+    <t>Kg de banana canaria</t>
+  </si>
+  <si>
+    <t>Pack 6L leche</t>
+  </si>
+  <si>
+    <t>Paquetes de azucar</t>
+  </si>
+  <si>
+    <t>CIF: U38230231</t>
+  </si>
+  <si>
+    <t>4 de marzo de 2026</t>
   </si>
 </sst>
 </file>
@@ -1265,12 +1254,12 @@
   <sheetData>
     <row r="1" spans="2:10" ht="61.15" customHeight="1">
       <c r="B1" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C1" s="6"/>
       <c r="D1" s="19"/>
       <c r="E1" s="19" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="2:10" ht="22.15" customHeight="1">
@@ -1278,10 +1267,10 @@
         <v>0</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E2" s="20">
         <v>3456</v>
@@ -1292,19 +1281,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D3" s="20" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" s="21">
-        <v>46085</v>
+        <v>11</v>
+      </c>
+      <c r="E3" s="21" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="2:10" ht="22.15" customHeight="1">
       <c r="B4" s="3"/>
       <c r="C4" s="3" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4" s="20"/>
       <c r="E4" s="21"/>
@@ -1322,38 +1311,22 @@
       <c r="E6" s="24"/>
     </row>
     <row r="7" spans="2:10" s="10" customFormat="1" ht="21" customHeight="1">
-      <c r="B7" s="25" t="s">
-        <v>2</v>
-      </c>
-      <c r="C7" s="26" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" s="25" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" s="27" t="s">
-        <v>6</v>
-      </c>
+      <c r="B7" s="25"/>
+      <c r="C7" s="26"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="27"/>
     </row>
     <row r="8" spans="2:10" ht="48" customHeight="1">
       <c r="B8" s="4"/>
-      <c r="C8" s="13" t="s">
-        <v>7</v>
-      </c>
+      <c r="C8" s="13"/>
       <c r="D8" s="12"/>
-      <c r="E8" s="16" t="s">
-        <v>7</v>
-      </c>
+      <c r="E8" s="16"/>
     </row>
     <row r="9" spans="2:10" ht="22.15" customHeight="1">
       <c r="B9" s="4"/>
-      <c r="C9" s="8" t="s">
-        <v>8</v>
-      </c>
+      <c r="C9" s="8"/>
       <c r="D9" s="12"/>
-      <c r="E9" s="17" t="s">
-        <v>8</v>
-      </c>
+      <c r="E9" s="17"/>
     </row>
     <row r="10" spans="2:10" ht="23.1" customHeight="1">
       <c r="B10" s="14"/>
@@ -1364,31 +1337,31 @@
     </row>
     <row r="11" spans="2:10" s="9" customFormat="1" ht="40.15" customHeight="1">
       <c r="B11" s="28" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C11" s="29" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D11" s="30" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="E11" s="31" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="2:10" ht="40.15" customHeight="1">
       <c r="B12" s="32">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D12" s="11">
-        <v>199.99</v>
+        <v>4.32</v>
       </c>
       <c r="E12" s="18">
         <f>IF(DetallesFactura[[#This Row],[PRECIO POR UNIDAD]]&lt;&gt;"",DetallesFactura[[#This Row],[CANT.]]*DetallesFactura[[#This Row],[PRECIO POR UNIDAD]],"")</f>
-        <v>399.98</v>
+        <v>4.32</v>
       </c>
     </row>
     <row r="13" spans="2:10" ht="40.15" customHeight="1">
@@ -1396,7 +1369,7 @@
         <v>2</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D13" s="11">
         <v>3.99</v>
@@ -1407,23 +1380,33 @@
       </c>
     </row>
     <row r="14" spans="2:10" ht="40.15" customHeight="1">
-      <c r="B14" s="32"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="18"/>
+      <c r="B14" s="32">
+        <v>1</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D14" s="11">
+        <v>6.55</v>
+      </c>
+      <c r="E14" s="18">
+        <f>IF(DetallesFactura[[#This Row],[PRECIO POR UNIDAD]]&lt;&gt;"",DetallesFactura[[#This Row],[CANT.]]*DetallesFactura[[#This Row],[PRECIO POR UNIDAD]],"")</f>
+        <v>6.55</v>
+      </c>
     </row>
     <row r="15" spans="2:10" ht="40.15" customHeight="1">
       <c r="B15" s="32">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D15" s="11">
-        <v>18.989999999999998</v>
+        <v>1.23</v>
       </c>
       <c r="E15" s="18">
         <f>IF(DetallesFactura[[#This Row],[PRECIO POR UNIDAD]]&lt;&gt;"",DetallesFactura[[#This Row],[CANT.]]*DetallesFactura[[#This Row],[PRECIO POR UNIDAD]],"")</f>
-        <v>18.989999999999998</v>
+        <v>3.69</v>
       </c>
     </row>
     <row r="16" spans="2:10" ht="40.15" customHeight="1">
@@ -1501,11 +1484,11 @@
     <row r="25" spans="2:5" ht="50.1" customHeight="1">
       <c r="B25" s="34" t="str">
         <f>"Todos los cheques se extenderán a nombre de "&amp; NombreEmpresa</f>
-        <v xml:space="preserve">Todos los cheques se extenderán a nombre de Juguetos </v>
+        <v>Todos los cheques se extenderán a nombre de Eroski</v>
       </c>
       <c r="C25" s="34"/>
       <c r="D25" s="35" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E25" s="40">
         <v>0.21</v>
@@ -1513,15 +1496,15 @@
     </row>
     <row r="26" spans="2:5" ht="50.1" customHeight="1">
       <c r="B26" s="36" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C26" s="37"/>
       <c r="D26" s="38" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E26" s="39">
         <f>SUM(E12:E24) * (1+E25)</f>
-        <v>516.60950000000003</v>
+        <v>27.273400000000002</v>
       </c>
     </row>
   </sheetData>
@@ -1578,15 +1561,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="26" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ac37c1753acd5e330d2062ccec26ea66">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3b340c7101c92c5120abd06486f94548" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -1886,6 +1860,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1907,14 +1890,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ACAD8A25-8121-4279-8C27-CB49DFB12BB5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C5EE937-CA2A-4DA3-9616-40EB800F3A39}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1935,6 +1910,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ACAD8A25-8121-4279-8C27-CB49DFB12BB5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{251985EC-1981-4124-91C1-072B1A12AD5C}">
   <ds:schemaRefs>

</xml_diff>